<commit_message>
update yaml file name
</commit_message>
<xml_diff>
--- a/src/aat/resources/adv_bundling_functional_tests_ccd_def.xlsx
+++ b/src/aat/resources/adv_bundling_functional_tests_ccd_def.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30224"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30306"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JAMIL\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="42" documentId="13_ncr:1_{D775BDB6-81C0-4A98-AE91-5EE12938AC55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB767CC0-6D52-49F2-AFD4-67EA8AB9AD5C}"/>
+  <xr:revisionPtr revIDLastSave="43" documentId="13_ncr:1_{D775BDB6-81C0-4A98-AE91-5EE12938AC55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{94A46562-413E-4D63-AD27-0C24BA2DEF67}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="19" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Change History" sheetId="1" r:id="rId1"/>
@@ -920,7 +920,7 @@
     <t>Tests - Config includes Watermark image</t>
   </si>
   <si>
-    <t>testbundleconfiguration/f-tests-14-subtitles-off.yaml</t>
+    <t>testbundleconfiguration/f-tests-14-subtitles-on.yaml</t>
   </si>
   <si>
     <t>Tests - Config disables Document Subtitles</t>

</xml_diff>